<commit_message>
Show current cash balances and publish English setup and usage guides
</commit_message>
<xml_diff>
--- a/examples/excel/robo_advisor_dashboard_demo.xlsx
+++ b/examples/excel/robo_advisor_dashboard_demo.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/1huang/Desktop/Robo Advisor /cuhk-cdas-robo-advisor/data/final/"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C207BF8-4F0D-3742-9291-3C923E008C4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>